<commit_message>
🚀 Prep for production: Added Procfile, production settings, and SEO metadata
</commit_message>
<xml_diff>
--- a/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
+++ b/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>535500</v>
+        <v>1088493</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="F2" t="n">
-        <v>535500</v>
+        <v>988493</v>
       </c>
     </row>
     <row r="3">
@@ -491,13 +491,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>50872.5</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>50872.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: resolve production 404s and implement financial logic safeguards
- Replace hardcoded localhost URLs with NEXT_PUBLIC_API_URL environment variable.\n- Add backend validation to prevent payments exceeding client debt.\n- Disable payment button in UI when debt is zero.\n- Add frontend validation for payment amounts.
</commit_message>
<xml_diff>
--- a/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
+++ b/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1088493</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>100000</v>
+        <v>400000</v>
       </c>
       <c r="F2" t="n">
-        <v>988493</v>
+        <v>-400000</v>
       </c>
     </row>
     <row r="3">
@@ -491,13 +491,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50872.5</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>50872.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: remove categories, enable client deletion, and fix debt logic
</commit_message>
<xml_diff>
--- a/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
+++ b/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>208250</v>
       </c>
       <c r="E2" t="n">
         <v>400000</v>
       </c>
       <c r="F2" t="n">
-        <v>-400000</v>
+        <v>-191750</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
feat: implement dark mode with persistence and UI toggle
</commit_message>
<xml_diff>
--- a/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
+++ b/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>208250</v>
+        <v>309400</v>
       </c>
       <c r="E2" t="n">
-        <v>400000</v>
+        <v>208750</v>
       </c>
       <c r="F2" t="n">
-        <v>-191750</v>
+        <v>100650</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Revert "feat: implement dark mode with persistence and UI toggle"
This reverts commit 5db224609a5bbf586cb816146aefc137e431a8d3.
</commit_message>
<xml_diff>
--- a/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
+++ b/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>309400</v>
+        <v>208250</v>
       </c>
       <c r="E2" t="n">
-        <v>208750</v>
+        <v>400000</v>
       </c>
       <c r="F2" t="n">
-        <v>100650</v>
+        <v>-191750</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
chore: update financial backup, trigger Vercel redeploy
Production frontend build verified (7 routes, all static).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
+++ b/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
@@ -468,10 +468,10 @@
         <v>208250</v>
       </c>
       <c r="E2" t="n">
-        <v>400000</v>
+        <v>608250</v>
       </c>
       <c r="F2" t="n">
-        <v>-191750</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
feat(stock): phase 1 - packaging inventory engine + per-order deduction
Product is now a liquid (alcohol_degree, price_per_liter, cost_per_liter,
stock_liters). Orders carry a FORMAT (carton 250/500/1L, bidon 5L, IBC,
vrac); each format maps to a bill of materials.

- formats.py: catalogue mapping format -> liters + packaging + labels
- OrderItem: format, liters (auto-computed), stock_applied lock
- Packaging: add Bidon type, carton sizes, per-degree labels, low-stock threshold
- signals: reserve stock on create, restore on CANCEL/delete, idempotent;
  totals computed per liter; debt still only on DELIVERED
- admin: edit new fields; serializers expose them; invoice/BL show format+liters

Verified end-to-end: create -> cancel -> reactivate -> delete all balance correctly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
+++ b/backend/AKRABIOLAB_FINANCIAL_BACKUP.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BENSELAMI nadir</t>
+          <t>TEST Client</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -461,42 +461,16 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0770394041</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>208250</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>608250</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ramzi</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Parfumerie</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0782235954</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>